<commit_message>
J3: preserve prepared sheet reference parity
</commit_message>
<xml_diff>
--- a/src/test/fixtures/xlsx/variant-comment-long-sheet.xlsx
+++ b/src/test/fixtures/xlsx/variant-comment-long-sheet.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commented worksheet with a very long name" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commented worksheet with a very long note" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="LongSheetCell">'Commented worksheet with a very long note'!$A$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -138,6 +140,20 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LongTable" displayName="LongTable" ref="A1:C5" headerRowCount="1">
+  <autoFilter ref="A1:C5"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Q"/>
+    <tableColumn id="2" name="V"/>
+    <tableColumn id="3" name="Linked">
+      <calculatedColumnFormula>'Commented worksheet with a very long note'!$A$1</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -429,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,6 +459,11 @@
           <t>V</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -453,6 +474,10 @@
       <c r="B2" t="n">
         <v>120</v>
       </c>
+      <c r="C2">
+        <f>'Commented worksheet with a very long note'!$A$1</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -463,6 +488,10 @@
       <c r="B3" t="n">
         <v>150</v>
       </c>
+      <c r="C3">
+        <f>'Commented worksheet with a very long note'!$A$1</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -473,6 +502,10 @@
       <c r="B4" t="n">
         <v>90</v>
       </c>
+      <c r="C4">
+        <f>'Commented worksheet with a very long note'!$A$1</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -482,11 +515,18 @@
       </c>
       <c r="B5" t="n">
         <v>200</v>
+      </c>
+      <c r="C5">
+        <f>'Commented worksheet with a very long note'!$A$1</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -498,7 +538,13 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>